<commit_message>
univava playoffs: quartas no site, com chave, premiacao e pesos
- 9 mapas das quartas (17 e 18/10): Golden 2x0 MackLogic Red, UFU 2x1 AXIS,
  CEUB 2x0 Turuna e CAAP 2x0 Wolf. Casados pelo PUUID do elenco inscrito no
  Challengermode: 5 de 5 em todo lado e nenhuma conta sem cadastro.
- Override univava-playoffs: eliminacao simples de 8, quartas e semis MD3
  online, final MD5 presencial, tier S, R$15.000, capa da fase de grupos.
  Em andamento: semis e final na chave sem placar, e so os eliminados das
  quartas com colocacao (5-8).
- ranking-weights: fase padrao playoffs e final na serie 7, como a AOC. Em
  andamento, o campeonato nao pontua.
- round_state_winrates recalculado com os mapas novos.

Ranking: so o corte de 20/10 muda (CAAP 5o->4o, MackLogic Red 4o->5o).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados_excel/round_state_winrates.xlsx
+++ b/dados_excel/round_state_winrates.xlsx
@@ -462,10 +462,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5164</v>
+        <v>5224</v>
       </c>
       <c r="C2" t="n">
-        <v>2582</v>
+        <v>2612</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>0.5</v>
@@ -478,13 +478,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6558</v>
+        <v>6632</v>
       </c>
       <c r="C3" t="n">
-        <v>1004</v>
+        <v>1016</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.1530954559316865</v>
+        <v>0.1531966224366707</v>
       </c>
     </row>
     <row r="4">
@@ -494,13 +494,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6911</v>
+        <v>6990</v>
       </c>
       <c r="C4" t="n">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.03574012443929966</v>
+        <v>0.03562231759656653</v>
       </c>
     </row>
     <row r="5">
@@ -510,13 +510,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5619</v>
+        <v>5678</v>
       </c>
       <c r="C5" t="n">
         <v>47</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.008364477665064958</v>
+        <v>0.008277562522014795</v>
       </c>
     </row>
     <row r="6">
@@ -526,13 +526,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2642</v>
+        <v>2668</v>
       </c>
       <c r="C6" t="n">
         <v>5</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.001892505677517033</v>
+        <v>0.001874062968515742</v>
       </c>
     </row>
     <row r="7">
@@ -542,13 +542,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6558</v>
+        <v>6632</v>
       </c>
       <c r="C7" t="n">
-        <v>5554</v>
+        <v>5616</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.8469045440683135</v>
+        <v>0.8468033775633294</v>
       </c>
     </row>
     <row r="8">
@@ -558,10 +558,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8026</v>
+        <v>8122</v>
       </c>
       <c r="C8" t="n">
-        <v>4013</v>
+        <v>4061</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>0.5</v>
@@ -574,13 +574,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8903</v>
+        <v>9011</v>
       </c>
       <c r="C9" t="n">
-        <v>1904</v>
+        <v>1928</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.2138604964618668</v>
+        <v>0.2139607146820553</v>
       </c>
     </row>
     <row r="10">
@@ -590,13 +590,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8124</v>
+        <v>8213</v>
       </c>
       <c r="C10" t="n">
-        <v>612</v>
+        <v>618</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.07533234859675036</v>
+        <v>0.07524656033118227</v>
       </c>
     </row>
     <row r="11">
@@ -606,13 +606,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4622</v>
+        <v>4672</v>
       </c>
       <c r="C11" t="n">
         <v>104</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.02250108178277802</v>
+        <v>0.02226027397260274</v>
       </c>
     </row>
     <row r="12">
@@ -622,13 +622,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6911</v>
+        <v>6990</v>
       </c>
       <c r="C12" t="n">
-        <v>6664</v>
+        <v>6741</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.9642598755607004</v>
+        <v>0.9643776824034335</v>
       </c>
     </row>
     <row r="13">
@@ -638,13 +638,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>8903</v>
+        <v>9011</v>
       </c>
       <c r="C13" t="n">
-        <v>6999</v>
+        <v>7083</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.7861395035381332</v>
+        <v>0.7860392853179448</v>
       </c>
     </row>
     <row r="14">
@@ -654,10 +654,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>10880</v>
+        <v>11018</v>
       </c>
       <c r="C14" t="n">
-        <v>5440</v>
+        <v>5509</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>0.5</v>
@@ -670,13 +670,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>11648</v>
+        <v>11783</v>
       </c>
       <c r="C15" t="n">
-        <v>3003</v>
+        <v>3041</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.2578125</v>
+        <v>0.25808367987779</v>
       </c>
     </row>
     <row r="16">
@@ -686,13 +686,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>8495</v>
+        <v>8587</v>
       </c>
       <c r="C16" t="n">
-        <v>930</v>
+        <v>939</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.1094761624484991</v>
+        <v>0.1093513450564807</v>
       </c>
     </row>
     <row r="17">
@@ -702,13 +702,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5619</v>
+        <v>5678</v>
       </c>
       <c r="C17" t="n">
-        <v>5572</v>
+        <v>5631</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.991635522334935</v>
+        <v>0.9917224374779852</v>
       </c>
     </row>
     <row r="18">
@@ -718,13 +718,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>8124</v>
+        <v>8213</v>
       </c>
       <c r="C18" t="n">
-        <v>7512</v>
+        <v>7595</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.9246676514032496</v>
+        <v>0.9247534396688177</v>
       </c>
     </row>
     <row r="19">
@@ -734,13 +734,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>11648</v>
+        <v>11783</v>
       </c>
       <c r="C19" t="n">
-        <v>8645</v>
+        <v>8742</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.7421875</v>
+        <v>0.74191632012221</v>
       </c>
     </row>
     <row r="20">
@@ -750,10 +750,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>15628</v>
+        <v>15814</v>
       </c>
       <c r="C20" t="n">
-        <v>7814</v>
+        <v>7907</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>0.5</v>
@@ -766,13 +766,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>16288</v>
+        <v>16473</v>
       </c>
       <c r="C21" t="n">
-        <v>4691</v>
+        <v>4736</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.2880034381139489</v>
+        <v>0.2875007588174588</v>
       </c>
     </row>
     <row r="22">
@@ -782,13 +782,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2642</v>
+        <v>2668</v>
       </c>
       <c r="C22" t="n">
-        <v>2637</v>
+        <v>2663</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.9981074943224829</v>
+        <v>0.9981259370314842</v>
       </c>
     </row>
     <row r="23">
@@ -798,13 +798,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>4622</v>
+        <v>4672</v>
       </c>
       <c r="C23" t="n">
-        <v>4518</v>
+        <v>4568</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.977498918217222</v>
+        <v>0.9777397260273972</v>
       </c>
     </row>
     <row r="24">
@@ -814,13 +814,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>8495</v>
+        <v>8587</v>
       </c>
       <c r="C24" t="n">
-        <v>7565</v>
+        <v>7648</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.8905238375515009</v>
+        <v>0.8906486549435193</v>
       </c>
     </row>
     <row r="25">
@@ -830,13 +830,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>16288</v>
+        <v>16473</v>
       </c>
       <c r="C25" t="n">
-        <v>11597</v>
+        <v>11737</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.7119965618860511</v>
+        <v>0.7124992411825412</v>
       </c>
     </row>
     <row r="26">
@@ -846,10 +846,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>32454</v>
+        <v>32826</v>
       </c>
       <c r="C26" t="n">
-        <v>16227</v>
+        <v>16413</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>0.5</v>

</xml_diff>

<commit_message>
copa luce: rodadas 5 a 7 e etapa 1 encerrada
- 9 mapas novos: P18 UFRJ Minerva 2x0 Shadows, P22 Wolf 2x1 Thunders,
  P24 A2E 2x0 Sheriff e P27 Wolf 2x0 A2E.
- 8 W.O., confirmados pelo dono: P17, P19, P20, P21, P23, P25, P26 e P28.
  Na plataforma, 13x0 lancado pelo admin nos dois mapas; nas matchlists dos
  inscritos, nenhuma partida entre as duas equipes.
- Tabela final da Etapa 1: Wolf 7-0, A2E 6-1, Thunders 5-2 e UFRJ Minerva
  4-3 classificadas; Shadows, Sheriff, Krakens e Artemis eliminadas, com
  colocacao de 5o a 8o. Semifinais em 01/11 e final em 07/11.
- round_state_winrates recalculado com os mapas novos.

Ranking: mudam so os cortes de 06, 13 e 20/10.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados_excel/round_state_winrates.xlsx
+++ b/dados_excel/round_state_winrates.xlsx
@@ -462,10 +462,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5224</v>
+        <v>5260</v>
       </c>
       <c r="C2" t="n">
-        <v>2612</v>
+        <v>2630</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>0.5</v>
@@ -478,13 +478,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6632</v>
+        <v>6701</v>
       </c>
       <c r="C3" t="n">
-        <v>1016</v>
+        <v>1023</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.1531966224366707</v>
+        <v>0.1526637815251455</v>
       </c>
     </row>
     <row r="4">
@@ -494,13 +494,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6990</v>
+        <v>7073</v>
       </c>
       <c r="C4" t="n">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.03562231759656653</v>
+        <v>0.03548706348084264</v>
       </c>
     </row>
     <row r="5">
@@ -510,13 +510,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5678</v>
+        <v>5734</v>
       </c>
       <c r="C5" t="n">
         <v>47</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.008277562522014795</v>
+        <v>0.00819672131147541</v>
       </c>
     </row>
     <row r="6">
@@ -526,13 +526,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2668</v>
+        <v>2697</v>
       </c>
       <c r="C6" t="n">
         <v>5</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.001874062968515742</v>
+        <v>0.001853911753800519</v>
       </c>
     </row>
     <row r="7">
@@ -542,13 +542,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6632</v>
+        <v>6701</v>
       </c>
       <c r="C7" t="n">
-        <v>5616</v>
+        <v>5678</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.8468033775633294</v>
+        <v>0.8473362184748545</v>
       </c>
     </row>
     <row r="8">
@@ -558,10 +558,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8122</v>
+        <v>8204</v>
       </c>
       <c r="C8" t="n">
-        <v>4061</v>
+        <v>4102</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>0.5</v>
@@ -574,13 +574,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9011</v>
+        <v>9112</v>
       </c>
       <c r="C9" t="n">
-        <v>1928</v>
+        <v>1949</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.2139607146820553</v>
+        <v>0.2138937664618086</v>
       </c>
     </row>
     <row r="10">
@@ -590,13 +590,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8213</v>
+        <v>8309</v>
       </c>
       <c r="C10" t="n">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.07524656033118227</v>
+        <v>0.07473823564809243</v>
       </c>
     </row>
     <row r="11">
@@ -606,13 +606,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4672</v>
+        <v>4728</v>
       </c>
       <c r="C11" t="n">
         <v>104</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.02226027397260274</v>
+        <v>0.02199661590524535</v>
       </c>
     </row>
     <row r="12">
@@ -622,13 +622,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6990</v>
+        <v>7073</v>
       </c>
       <c r="C12" t="n">
-        <v>6741</v>
+        <v>6822</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.9643776824034335</v>
+        <v>0.9645129365191574</v>
       </c>
     </row>
     <row r="13">
@@ -638,13 +638,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>9011</v>
+        <v>9112</v>
       </c>
       <c r="C13" t="n">
-        <v>7083</v>
+        <v>7163</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.7860392853179448</v>
+        <v>0.7861062335381914</v>
       </c>
     </row>
     <row r="14">
@@ -654,10 +654,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>11018</v>
+        <v>11126</v>
       </c>
       <c r="C14" t="n">
-        <v>5509</v>
+        <v>5563</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>0.5</v>
@@ -670,13 +670,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>11783</v>
+        <v>11906</v>
       </c>
       <c r="C15" t="n">
-        <v>3041</v>
+        <v>3068</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.25808367987779</v>
+        <v>0.2576852007391232</v>
       </c>
     </row>
     <row r="16">
@@ -686,13 +686,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>8587</v>
+        <v>8684</v>
       </c>
       <c r="C16" t="n">
-        <v>939</v>
+        <v>946</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.1093513450564807</v>
+        <v>0.1089359742054353</v>
       </c>
     </row>
     <row r="17">
@@ -702,13 +702,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5678</v>
+        <v>5734</v>
       </c>
       <c r="C17" t="n">
-        <v>5631</v>
+        <v>5687</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.9917224374779852</v>
+        <v>0.9918032786885246</v>
       </c>
     </row>
     <row r="18">
@@ -718,13 +718,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>8213</v>
+        <v>8309</v>
       </c>
       <c r="C18" t="n">
-        <v>7595</v>
+        <v>7688</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.9247534396688177</v>
+        <v>0.9252617643519075</v>
       </c>
     </row>
     <row r="19">
@@ -734,13 +734,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>11783</v>
+        <v>11906</v>
       </c>
       <c r="C19" t="n">
-        <v>8742</v>
+        <v>8838</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.74191632012221</v>
+        <v>0.7423147992608768</v>
       </c>
     </row>
     <row r="20">
@@ -750,10 +750,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>15814</v>
+        <v>15978</v>
       </c>
       <c r="C20" t="n">
-        <v>7907</v>
+        <v>7989</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>0.5</v>
@@ -766,13 +766,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>16473</v>
+        <v>16652</v>
       </c>
       <c r="C21" t="n">
-        <v>4736</v>
+        <v>4784</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.2875007588174588</v>
+        <v>0.287292817679558</v>
       </c>
     </row>
     <row r="22">
@@ -782,13 +782,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2668</v>
+        <v>2697</v>
       </c>
       <c r="C22" t="n">
-        <v>2663</v>
+        <v>2692</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.9981259370314842</v>
+        <v>0.9981460882461994</v>
       </c>
     </row>
     <row r="23">
@@ -798,13 +798,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>4672</v>
+        <v>4728</v>
       </c>
       <c r="C23" t="n">
-        <v>4568</v>
+        <v>4624</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.9777397260273972</v>
+        <v>0.9780033840947546</v>
       </c>
     </row>
     <row r="24">
@@ -814,13 +814,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>8587</v>
+        <v>8684</v>
       </c>
       <c r="C24" t="n">
-        <v>7648</v>
+        <v>7738</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.8906486549435193</v>
+        <v>0.8910640257945647</v>
       </c>
     </row>
     <row r="25">
@@ -830,13 +830,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>16473</v>
+        <v>16652</v>
       </c>
       <c r="C25" t="n">
-        <v>11737</v>
+        <v>11868</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.7124992411825412</v>
+        <v>0.7127071823204419</v>
       </c>
     </row>
     <row r="26">
@@ -846,10 +846,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>32826</v>
+        <v>33184</v>
       </c>
       <c r="C26" t="n">
-        <v>16413</v>
+        <v>16592</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>0.5</v>

</xml_diff>

<commit_message>
univava playoffs: semifinais no site
- 4 mapas das semis (24/10): Golden 2x0 UFU Saints (Ascent 13-7, Split 13-8)
  e CEUB Octopus 2x0 CAAP Hellhounds (Summit 13-3, Haven 13-8). Coletados com
  o PegaTeamMatch por confronto direto; 20 de 20 jogadores casados pelo PUUID
  do cadastro. A CEUB da semi e a Octopus (5 de 5 do elenco), nao a Vulgaris.
- Um Ascent reiniciado (13:59, 3x1, sem vencedor) ficou de fora pelo filtro
  de 13 rounds; o mapa valido comecou as 14:16.
- Override: placar nas P5 e P6, final P7 Golden x CEUB Octopus, UFU e CAAP
  em 3-4. Segue em andamento ate a final.
- round_state_winrates recalculado com os mapas novos.
- team-profiles.json estava atrasado desde o checkpoint de 23/10 (37 equipes
  mudam so por isso); os mapas novos mexem apenas nas 4 equipes das semis,
  medido contra o build com as entradas do HEAD.

Ranking: nenhuma posicao muda nos 41 cortes; a nota varia no maximo 0,001.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados_excel/round_state_winrates.xlsx
+++ b/dados_excel/round_state_winrates.xlsx
@@ -430,7 +430,7 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -462,10 +462,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5364</v>
+        <v>5380</v>
       </c>
       <c r="C2" t="n">
-        <v>2682</v>
+        <v>2690</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>0.5</v>
@@ -478,13 +478,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6824</v>
+        <v>6849</v>
       </c>
       <c r="C3" t="n">
-        <v>1041</v>
+        <v>1046</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.1525498241500586</v>
+        <v>0.1527230252591619</v>
       </c>
     </row>
     <row r="4">
@@ -494,13 +494,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7226</v>
+        <v>7256</v>
       </c>
       <c r="C4" t="n">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.03556601162468862</v>
+        <v>0.03555678059536935</v>
       </c>
     </row>
     <row r="5">
@@ -510,13 +510,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5851</v>
+        <v>5879</v>
       </c>
       <c r="C5" t="n">
         <v>49</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.008374636814219792</v>
+        <v>0.008334750807960537</v>
       </c>
     </row>
     <row r="6">
@@ -526,13 +526,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2747</v>
+        <v>2759</v>
       </c>
       <c r="C6" t="n">
         <v>6</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.002184200946487077</v>
+        <v>0.00217470097861544</v>
       </c>
     </row>
     <row r="7">
@@ -542,13 +542,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6824</v>
+        <v>6849</v>
       </c>
       <c r="C7" t="n">
-        <v>5783</v>
+        <v>5803</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.8474501758499414</v>
+        <v>0.8472769747408381</v>
       </c>
     </row>
     <row r="8">
@@ -558,10 +558,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8356</v>
+        <v>8390</v>
       </c>
       <c r="C8" t="n">
-        <v>4178</v>
+        <v>4195</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>0.5</v>
@@ -574,13 +574,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9290</v>
+        <v>9328</v>
       </c>
       <c r="C9" t="n">
-        <v>1983</v>
+        <v>1987</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.2134553283100108</v>
+        <v>0.2130145797598628</v>
       </c>
     </row>
     <row r="10">
@@ -590,13 +590,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8494</v>
+        <v>8533</v>
       </c>
       <c r="C10" t="n">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.0744054626795385</v>
+        <v>0.07429977733505215</v>
       </c>
     </row>
     <row r="11">
@@ -606,13 +606,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4825</v>
+        <v>4848</v>
       </c>
       <c r="C11" t="n">
         <v>105</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.02176165803108808</v>
+        <v>0.02165841584158416</v>
       </c>
     </row>
     <row r="12">
@@ -622,13 +622,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7226</v>
+        <v>7256</v>
       </c>
       <c r="C12" t="n">
-        <v>6969</v>
+        <v>6998</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.9644339883753114</v>
+        <v>0.9644432194046306</v>
       </c>
     </row>
     <row r="13">
@@ -638,13 +638,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>9290</v>
+        <v>9328</v>
       </c>
       <c r="C13" t="n">
-        <v>7307</v>
+        <v>7341</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.7865446716899892</v>
+        <v>0.7869854202401372</v>
       </c>
     </row>
     <row r="14">
@@ -654,10 +654,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>11316</v>
+        <v>11360</v>
       </c>
       <c r="C14" t="n">
-        <v>5658</v>
+        <v>5680</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>0.5</v>
@@ -670,13 +670,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>12139</v>
+        <v>12190</v>
       </c>
       <c r="C15" t="n">
-        <v>3123</v>
+        <v>3136</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.2572699563390724</v>
+        <v>0.2572600492206727</v>
       </c>
     </row>
     <row r="16">
@@ -686,13 +686,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>8856</v>
+        <v>8903</v>
       </c>
       <c r="C16" t="n">
-        <v>967</v>
+        <v>970</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.1091915085817525</v>
+        <v>0.1089520386386611</v>
       </c>
     </row>
     <row r="17">
@@ -702,13 +702,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5851</v>
+        <v>5879</v>
       </c>
       <c r="C17" t="n">
-        <v>5802</v>
+        <v>5830</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.9916253631857802</v>
+        <v>0.9916652491920395</v>
       </c>
     </row>
     <row r="18">
@@ -718,13 +718,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>8494</v>
+        <v>8533</v>
       </c>
       <c r="C18" t="n">
-        <v>7862</v>
+        <v>7899</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.9255945373204615</v>
+        <v>0.9257002226649479</v>
       </c>
     </row>
     <row r="19">
@@ -734,13 +734,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>12139</v>
+        <v>12190</v>
       </c>
       <c r="C19" t="n">
-        <v>9016</v>
+        <v>9054</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.7427300436609275</v>
+        <v>0.7427399507793273</v>
       </c>
     </row>
     <row r="20">
@@ -750,10 +750,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>16294</v>
+        <v>16348</v>
       </c>
       <c r="C20" t="n">
-        <v>8147</v>
+        <v>8174</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>0.5</v>
@@ -766,13 +766,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>16982</v>
+        <v>17056</v>
       </c>
       <c r="C21" t="n">
-        <v>4880</v>
+        <v>4896</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.2873630903309387</v>
+        <v>0.2870544090056285</v>
       </c>
     </row>
     <row r="22">
@@ -782,13 +782,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2747</v>
+        <v>2759</v>
       </c>
       <c r="C22" t="n">
-        <v>2741</v>
+        <v>2753</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.9978157990535129</v>
+        <v>0.9978252990213845</v>
       </c>
     </row>
     <row r="23">
@@ -798,13 +798,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>4825</v>
+        <v>4848</v>
       </c>
       <c r="C23" t="n">
-        <v>4720</v>
+        <v>4743</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.9782383419689119</v>
+        <v>0.9783415841584159</v>
       </c>
     </row>
     <row r="24">
@@ -814,13 +814,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>8856</v>
+        <v>8903</v>
       </c>
       <c r="C24" t="n">
-        <v>7889</v>
+        <v>7933</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.8908084914182475</v>
+        <v>0.8910479613613389</v>
       </c>
     </row>
     <row r="25">
@@ -830,13 +830,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>16982</v>
+        <v>17056</v>
       </c>
       <c r="C25" t="n">
-        <v>12102</v>
+        <v>12160</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.7126369096690613</v>
+        <v>0.7129455909943715</v>
       </c>
     </row>
     <row r="26">
@@ -846,10 +846,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>33844</v>
+        <v>34000</v>
       </c>
       <c r="C26" t="n">
-        <v>16922</v>
+        <v>17000</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>0.5</v>

</xml_diff>